<commit_message>
bugfix e integrato readme
</commit_message>
<xml_diff>
--- a/output_ptf_delta.xlsx
+++ b/output_ptf_delta.xlsx
@@ -2211,7 +2211,7 @@
         <v>43899</v>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>1072.112381433874</v>
       </c>
       <c r="C47" t="n">
         <v>0</v>
@@ -2220,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>-90.7338890526657</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -2235,13 +2235,13 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>-989.3377101809991</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>7.959217799790265</v>
       </c>
     </row>
     <row r="48">
@@ -10267,7 +10267,7 @@
         <v>44204</v>
       </c>
       <c r="B259" t="n">
-        <v>0</v>
+        <v>-1259.103425426237</v>
       </c>
       <c r="C259" t="n">
         <v>0</v>
@@ -10276,7 +10276,7 @@
         <v>0</v>
       </c>
       <c r="E259" t="n">
-        <v>0</v>
+        <v>130.5690577088668</v>
       </c>
       <c r="F259" t="n">
         <v>0</v>
@@ -10291,13 +10291,13 @@
         <v>0</v>
       </c>
       <c r="J259" t="n">
-        <v>0</v>
+        <v>1033.000598829424</v>
       </c>
       <c r="K259" t="n">
         <v>0</v>
       </c>
       <c r="L259" t="n">
-        <v>0</v>
+        <v>95.53376888794693</v>
       </c>
     </row>
     <row r="260">
@@ -34739,7 +34739,7 @@
         <v>45140</v>
       </c>
       <c r="B903" t="n">
-        <v>0</v>
+        <v>-908.741779095761</v>
       </c>
       <c r="C903" t="n">
         <v>0</v>
@@ -34748,7 +34748,7 @@
         <v>0</v>
       </c>
       <c r="E903" t="n">
-        <v>0</v>
+        <v>-104.2624286171507</v>
       </c>
       <c r="F903" t="n">
         <v>0</v>
@@ -34763,13 +34763,13 @@
         <v>0</v>
       </c>
       <c r="J903" t="n">
-        <v>0</v>
+        <v>1194.45828075616</v>
       </c>
       <c r="K903" t="n">
         <v>0</v>
       </c>
       <c r="L903" t="n">
-        <v>0</v>
+        <v>-181.454073043247</v>
       </c>
     </row>
     <row r="904">

</xml_diff>